<commit_message>
Fix customer onboarding inputs, storage checks and deployment guidance (#237)
Co-authored-by: Mukesh Dua <mukeshdua+microsoft@microsoft.com>
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/utilities/onboarding-tool/scripts/stage1-planning/discovery-resource-planning-form-managed-vnet.xlsx
+++ b/utilities/onboarding-tool/scripts/stage1-planning/discovery-resource-planning-form-managed-vnet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\discovery-tool\discovery\utilities\onboarding-tool\scripts\stage1-planning\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\discovery\discovery\utilities\onboarding-tool\scripts\stage1-planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEDADC8E-B9E0-406E-81B2-A565DE0734AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6795" yWindow="2595" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -310,19 +310,19 @@
     <t>byo</t>
   </si>
   <si>
-    <t>byo | managed. Bookshelf (bookshelf.inScope=true) requires byo with storage.account set.</t>
+    <t>Must be byo. Every Discovery project needs a storage account you own; managed is not supported.</t>
   </si>
   <si>
     <t>storage.account</t>
   </si>
   <si>
-    <t>Name of the storage account you pre-created for project data (required, byo). The tool does not create it; Stage 1 checks that it exists.</t>
+    <t>Required. Name (not resource ID) of an existing StorageV2 account in the target subscription. The tool does not create it. Create one with: az storage account create -g &lt;rg&gt; -n &lt;globally-unique-name&gt; -l &lt;region&gt; --sku Standard_LRS --kind StorageV2 --min-tls-version TLS1_2 --allow-blob-public-access false. Stage 1 checks that it exists.</t>
   </si>
   <si>
     <t>storage.access</t>
   </si>
   <si>
-    <t>BYO storage network access: privateEndpoint | serviceEndpoint (default privateEndpoint). Ignored when storage.model=managed.</t>
+    <t>Storage network access: privateEndpoint | serviceEndpoint (default privateEndpoint).</t>
   </si>
   <si>
     <t>SIZING &amp; SCALE</t>
@@ -1430,15 +1430,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1742,7 +1742,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E65"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -1751,7 +1751,7 @@
     <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.45" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -1759,7 +1759,7 @@
       <c r="C1" s="15"/>
       <c r="D1" s="15"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
@@ -1767,7 +1767,7 @@
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
     </row>
-    <row r="4" spans="1:5" ht="58.3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>2</v>
       </c>
@@ -1782,7 +1782,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
         <v>6</v>
       </c>
@@ -1791,7 +1791,7 @@
       <c r="D5" s="15"/>
       <c r="E5" s="15"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>7</v>
       </c>
@@ -1802,7 +1802,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="25.75" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>10</v>
       </c>
@@ -1813,7 +1813,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="36" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:5" ht="48" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -1824,7 +1824,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>16</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>19</v>
       </c>
@@ -1846,7 +1846,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>22</v>
       </c>
@@ -1857,7 +1857,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="48" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:5" ht="48" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>24</v>
       </c>
@@ -1868,7 +1868,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>26</v>
       </c>
@@ -1879,7 +1879,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="25.75" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>29</v>
       </c>
@@ -1890,7 +1890,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="51.45" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:5" ht="51" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>32</v>
       </c>
@@ -1901,7 +1901,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>35</v>
       </c>
@@ -1910,7 +1910,7 @@
       <c r="D17" s="15"/>
       <c r="E17" s="15"/>
     </row>
-    <row r="18" spans="1:5" ht="24" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:5" ht="24" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
         <v>36</v>
       </c>
@@ -1921,7 +1921,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:5" ht="24" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
         <v>39</v>
       </c>
@@ -1932,7 +1932,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="24" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:5" ht="24" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
         <v>42</v>
       </c>
@@ -1941,7 +1941,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
         <v>44</v>
       </c>
@@ -1952,7 +1952,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
         <v>47</v>
       </c>
@@ -1963,7 +1963,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
         <v>49</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
         <v>51</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="24" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:5" ht="24" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
         <v>54</v>
       </c>
@@ -1994,12 +1994,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="10"/>
       <c r="B26" s="11"/>
       <c r="E26" s="12"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
         <v>57</v>
       </c>
@@ -2008,7 +2008,7 @@
       <c r="D28" s="15"/>
       <c r="E28" s="15"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
         <v>58</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
         <v>58</v>
       </c>
@@ -2042,7 +2042,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
         <v>58</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
         <v>58</v>
       </c>
@@ -2076,7 +2076,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
         <v>58</v>
       </c>
@@ -2093,7 +2093,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
         <v>58</v>
       </c>
@@ -2110,7 +2110,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
         <v>58</v>
       </c>
@@ -2127,7 +2127,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="16" t="s">
         <v>78</v>
       </c>
@@ -2136,7 +2136,7 @@
       <c r="D37" s="15"/>
       <c r="E37" s="15"/>
     </row>
-    <row r="38" spans="1:5" ht="24" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:5" ht="24" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
         <v>79</v>
       </c>
@@ -2147,7 +2147,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="24" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
         <v>82</v>
       </c>
@@ -2156,7 +2156,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="24" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:5" ht="24" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
         <v>84</v>
       </c>
@@ -2165,7 +2165,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
         <v>86</v>
       </c>
@@ -2174,7 +2174,7 @@
       <c r="D42" s="15"/>
       <c r="E42" s="15"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
         <v>87</v>
       </c>
@@ -2185,7 +2185,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
         <v>90</v>
       </c>
@@ -2196,7 +2196,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
         <v>92</v>
       </c>
@@ -2207,7 +2207,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
         <v>95</v>
       </c>
@@ -2218,7 +2218,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="24" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:5" ht="24" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
         <v>98</v>
       </c>
@@ -2227,7 +2227,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="24" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:5" ht="24" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
         <v>100</v>
       </c>
@@ -2238,7 +2238,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="16" t="s">
         <v>103</v>
       </c>
@@ -2247,7 +2247,7 @@
       <c r="D49" s="15"/>
       <c r="E49" s="15"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
         <v>104</v>
       </c>
@@ -2258,7 +2258,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
         <v>107</v>
       </c>
@@ -2269,7 +2269,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
         <v>110</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
         <v>113</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
         <v>115</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
         <v>117</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
         <v>120</v>
       </c>
@@ -2324,7 +2324,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
         <v>122</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="24" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:5" ht="24" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
         <v>124</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="16" t="s">
         <v>126</v>
       </c>
@@ -2353,20 +2353,20 @@
       <c r="D60" s="15"/>
       <c r="E60" s="15"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="13" t="s">
         <v>127</v>
       </c>
       <c r="B61" s="11"/>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
         <v>127</v>
       </c>
       <c r="B62" s="11"/>
       <c r="E62" s="12"/>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="16" t="s">
         <v>128</v>
       </c>
@@ -2375,7 +2375,7 @@
       <c r="D64" s="15"/>
       <c r="E64" s="15"/>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="13" t="s">
         <v>129</v>
       </c>
@@ -2396,7 +2396,7 @@
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A17:E17"/>
   </mergeCells>
-  <dataValidations count="10">
+  <dataValidations count="11">
     <dataValidation type="list" allowBlank="1" sqref="B9" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"devtest,prod"</formula1>
     </dataValidation>
@@ -2407,10 +2407,10 @@
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B18" xr:uid="{00000000-0002-0000-0000-000003000000}">
-      <formula1>"managed,byo-existing,byo,byo-spoke,greenfield"</formula1>
+      <formula1>"managed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B38" xr:uid="{00000000-0002-0000-0000-000004000000}">
-      <formula1>"byo,managed"</formula1>
+      <formula1>"byo"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="E29 E30 E31 E32 E33 E34 E35" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Microsoft.App/environments,Microsoft.ContainerService/managedClusters,none"</formula1>
@@ -2427,6 +2427,9 @@
     <dataValidation type="list" allowBlank="1" sqref="B48" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Enabled,Disabled"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B25" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+      <formula1>"UserDefinedRouting,LoadBalancer"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="rId1"/>
@@ -2436,26 +2439,26 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:C20"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="95" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="26.15" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="2" spans="2:3" ht="26.1" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="19" t="s">
         <v>130</v>
       </c>
       <c r="C2" s="15"/>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B3" s="18" t="s">
         <v>131</v>
       </c>
       <c r="C3" s="15"/>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>132</v>
       </c>
@@ -2463,7 +2466,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>134</v>
       </c>
@@ -2471,7 +2474,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>136</v>
       </c>
@@ -2479,7 +2482,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>138</v>
       </c>
@@ -2487,7 +2490,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>140</v>
       </c>
@@ -2495,7 +2498,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>142</v>
       </c>
@@ -2503,7 +2506,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>143</v>
       </c>
@@ -2511,7 +2514,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>144</v>
       </c>
@@ -2519,7 +2522,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>146</v>
       </c>
@@ -2527,7 +2530,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>147</v>
       </c>
@@ -2535,12 +2538,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="16" spans="2:3" ht="16.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:3" ht="16.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
         <v>150</v>
       </c>
@@ -2548,7 +2551,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>152</v>
       </c>
@@ -2556,7 +2559,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>154</v>
       </c>
@@ -2564,7 +2567,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
         <v>156</v>
       </c>
@@ -2584,9 +2587,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" ht="23.15" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:8" ht="23.1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="20" t="s">
         <v>158</v>
       </c>
@@ -2598,7 +2601,7 @@
       <c r="G1" s="15"/>
       <c r="H1" s="15"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>159</v>
       </c>
@@ -2622,7 +2625,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
@@ -2631,8 +2634,8 @@
     <col min="7" max="7" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="25" t="s">
         <v>160</v>
       </c>
       <c r="B1" s="15"/>
@@ -2642,7 +2645,7 @@
       <c r="F1" s="15"/>
       <c r="G1" s="15"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>161</v>
       </c>
@@ -2653,7 +2656,7 @@
       <c r="F2" s="15"/>
       <c r="G2" s="15"/>
     </row>
-    <row r="4" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>162</v>
       </c>
@@ -2666,7 +2669,7 @@
       <c r="F4" s="23"/>
       <c r="G4" s="24"/>
     </row>
-    <row r="5" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>144</v>
       </c>
@@ -2679,7 +2682,7 @@
       <c r="F5" s="23"/>
       <c r="G5" s="24"/>
     </row>
-    <row r="6" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>164</v>
       </c>
@@ -2692,7 +2695,7 @@
       <c r="F6" s="23"/>
       <c r="G6" s="24"/>
     </row>
-    <row r="7" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>166</v>
       </c>
@@ -2705,7 +2708,7 @@
       <c r="F7" s="23"/>
       <c r="G7" s="24"/>
     </row>
-    <row r="8" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>168</v>
       </c>
@@ -2718,7 +2721,7 @@
       <c r="F8" s="23"/>
       <c r="G8" s="24"/>
     </row>
-    <row r="9" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>170</v>
       </c>
@@ -2731,8 +2734,8 @@
       <c r="F9" s="23"/>
       <c r="G9" s="24"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A11" s="25" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B11" s="15"/>
@@ -2742,7 +2745,7 @@
       <c r="F11" s="15"/>
       <c r="G11" s="15"/>
     </row>
-    <row r="12" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>173</v>
       </c>
@@ -2765,7 +2768,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>179</v>
       </c>
@@ -2788,7 +2791,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>184</v>
       </c>
@@ -2811,7 +2814,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>189</v>
       </c>
@@ -2834,7 +2837,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>73</v>
       </c>
@@ -2857,7 +2860,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="38.6" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" ht="38.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>75</v>
       </c>
@@ -2880,7 +2883,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>197</v>
       </c>
@@ -2903,7 +2906,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>204</v>
       </c>
@@ -2926,7 +2929,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>207</v>
       </c>
@@ -2949,7 +2952,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -2958,7 +2961,7 @@
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -2967,7 +2970,7 @@
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -2976,7 +2979,7 @@
       <c r="F23" s="8"/>
       <c r="G23" s="8"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -2985,7 +2988,7 @@
       <c r="F24" s="8"/>
       <c r="G24" s="8"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="8"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -2994,7 +2997,7 @@
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -3027,7 +3030,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -3038,8 +3041,8 @@
     <col min="8" max="8" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="25" t="s">
         <v>213</v>
       </c>
       <c r="B1" s="15"/>
@@ -3050,7 +3053,7 @@
       <c r="G1" s="15"/>
       <c r="H1" s="15"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>214</v>
       </c>
@@ -3062,7 +3065,7 @@
       <c r="G2" s="15"/>
       <c r="H2" s="15"/>
     </row>
-    <row r="4" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>215</v>
       </c>
@@ -3088,7 +3091,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:8" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>221</v>
       </c>
@@ -3114,7 +3117,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>229</v>
       </c>
@@ -3140,7 +3143,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>236</v>
       </c>
@@ -3166,7 +3169,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>241</v>
       </c>
@@ -3192,7 +3195,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:8" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>248</v>
       </c>
@@ -3218,7 +3221,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:8" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>254</v>
       </c>
@@ -3244,7 +3247,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:8" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>258</v>
       </c>
@@ -3270,7 +3273,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>263</v>
       </c>
@@ -3296,7 +3299,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -3306,7 +3309,7 @@
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -3316,7 +3319,7 @@
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -3326,7 +3329,7 @@
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -3336,7 +3339,7 @@
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -3346,7 +3349,7 @@
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -3373,7 +3376,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -3384,8 +3387,8 @@
     <col min="8" max="8" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="25" t="s">
         <v>269</v>
       </c>
       <c r="B1" s="15"/>
@@ -3396,7 +3399,7 @@
       <c r="G1" s="15"/>
       <c r="H1" s="15"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>270</v>
       </c>
@@ -3408,8 +3411,8 @@
       <c r="G2" s="15"/>
       <c r="H2" s="15"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A4" s="25" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="21" t="s">
         <v>180</v>
       </c>
       <c r="B4" s="15"/>
@@ -3420,7 +3423,7 @@
       <c r="G4" s="15"/>
       <c r="H4" s="15"/>
     </row>
-    <row r="5" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>271</v>
       </c>
@@ -3440,7 +3443,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:8" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>179</v>
       </c>
@@ -3460,8 +3463,8 @@
         <v>278</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A8" s="25" t="s">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="21" t="s">
         <v>279</v>
       </c>
       <c r="B8" s="15"/>
@@ -3472,7 +3475,7 @@
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
     </row>
-    <row r="9" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>280</v>
       </c>
@@ -3498,7 +3501,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:8" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>59</v>
       </c>
@@ -3524,7 +3527,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:8" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>63</v>
       </c>
@@ -3550,7 +3553,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:8" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>65</v>
       </c>
@@ -3576,7 +3579,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:8" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>68</v>
       </c>
@@ -3602,7 +3605,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:8" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>70</v>
       </c>
@@ -3628,7 +3631,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="38.6" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:8" ht="38.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>73</v>
       </c>
@@ -3654,7 +3657,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="38.6" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:8" ht="38.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>75</v>
       </c>
@@ -3680,7 +3683,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -3690,7 +3693,7 @@
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -3700,7 +3703,7 @@
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="8"/>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -3710,7 +3713,7 @@
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -3720,7 +3723,7 @@
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -3744,7 +3747,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:L74"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
@@ -3759,8 +3762,8 @@
     <col min="11" max="11" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="25" t="s">
         <v>308</v>
       </c>
       <c r="B1" s="15"/>
@@ -3775,7 +3778,7 @@
       <c r="K1" s="15"/>
       <c r="L1" s="15"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>309</v>
       </c>
@@ -3791,7 +3794,7 @@
       <c r="K2" s="15"/>
       <c r="L2" s="15"/>
     </row>
-    <row r="4" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>310</v>
       </c>
@@ -3826,7 +3829,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>288</v>
       </c>
@@ -3861,7 +3864,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:12" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>288</v>
       </c>
@@ -3896,7 +3899,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>288</v>
       </c>
@@ -3931,7 +3934,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>288</v>
       </c>
@@ -3966,7 +3969,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>288</v>
       </c>
@@ -4001,7 +4004,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>288</v>
       </c>
@@ -4036,7 +4039,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:12" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>288</v>
       </c>
@@ -4071,7 +4074,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>288</v>
       </c>
@@ -4106,7 +4109,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>288</v>
       </c>
@@ -4141,7 +4144,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>288</v>
       </c>
@@ -4176,7 +4179,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:12" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>292</v>
       </c>
@@ -4211,7 +4214,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:12" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>292</v>
       </c>
@@ -4246,7 +4249,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>292</v>
       </c>
@@ -4281,7 +4284,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>292</v>
       </c>
@@ -4316,7 +4319,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>292</v>
       </c>
@@ -4351,7 +4354,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>292</v>
       </c>
@@ -4386,7 +4389,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>292</v>
       </c>
@@ -4421,7 +4424,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>292</v>
       </c>
@@ -4456,7 +4459,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>292</v>
       </c>
@@ -4491,7 +4494,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>292</v>
       </c>
@@ -4526,7 +4529,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>295</v>
       </c>
@@ -4561,7 +4564,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>295</v>
       </c>
@@ -4596,7 +4599,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>295</v>
       </c>
@@ -4631,7 +4634,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>295</v>
       </c>
@@ -4666,7 +4669,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>295</v>
       </c>
@@ -4701,7 +4704,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>295</v>
       </c>
@@ -4736,7 +4739,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>295</v>
       </c>
@@ -4771,7 +4774,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>295</v>
       </c>
@@ -4806,7 +4809,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>295</v>
       </c>
@@ -4841,7 +4844,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>295</v>
       </c>
@@ -4876,7 +4879,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>298</v>
       </c>
@@ -4911,7 +4914,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>298</v>
       </c>
@@ -4946,7 +4949,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>298</v>
       </c>
@@ -4981,7 +4984,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>298</v>
       </c>
@@ -5016,7 +5019,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>298</v>
       </c>
@@ -5051,7 +5054,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>298</v>
       </c>
@@ -5086,7 +5089,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>298</v>
       </c>
@@ -5121,7 +5124,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>298</v>
       </c>
@@ -5156,7 +5159,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>298</v>
       </c>
@@ -5191,7 +5194,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>298</v>
       </c>
@@ -5226,7 +5229,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>300</v>
       </c>
@@ -5261,7 +5264,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>300</v>
       </c>
@@ -5296,7 +5299,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>300</v>
       </c>
@@ -5331,7 +5334,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>300</v>
       </c>
@@ -5366,7 +5369,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>300</v>
       </c>
@@ -5401,7 +5404,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>300</v>
       </c>
@@ -5436,7 +5439,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>300</v>
       </c>
@@ -5471,7 +5474,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>300</v>
       </c>
@@ -5506,7 +5509,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>300</v>
       </c>
@@ -5541,7 +5544,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>300</v>
       </c>
@@ -5576,7 +5579,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>302</v>
       </c>
@@ -5611,7 +5614,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>302</v>
       </c>
@@ -5646,7 +5649,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>302</v>
       </c>
@@ -5681,7 +5684,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>302</v>
       </c>
@@ -5716,7 +5719,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>302</v>
       </c>
@@ -5751,7 +5754,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>302</v>
       </c>
@@ -5786,7 +5789,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>302</v>
       </c>
@@ -5821,7 +5824,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>302</v>
       </c>
@@ -5856,7 +5859,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>302</v>
       </c>
@@ -5891,7 +5894,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>302</v>
       </c>
@@ -5926,7 +5929,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>306</v>
       </c>
@@ -5961,7 +5964,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>306</v>
       </c>
@@ -5996,7 +5999,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>306</v>
       </c>
@@ -6031,7 +6034,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>306</v>
       </c>
@@ -6066,7 +6069,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>306</v>
       </c>
@@ -6101,7 +6104,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>306</v>
       </c>
@@ -6136,7 +6139,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="25.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:11" ht="25.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>306</v>
       </c>
@@ -6171,7 +6174,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>306</v>
       </c>
@@ -6206,7 +6209,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>306</v>
       </c>
@@ -6241,7 +6244,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>306</v>
       </c>
@@ -6299,7 +6302,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
@@ -6307,8 +6310,8 @@
     <col min="5" max="5" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="25" t="s">
         <v>342</v>
       </c>
       <c r="B1" s="15"/>
@@ -6317,7 +6320,7 @@
       <c r="E1" s="15"/>
       <c r="F1" s="15"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>343</v>
       </c>
@@ -6327,8 +6330,8 @@
       <c r="E2" s="15"/>
       <c r="F2" s="15"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A4" s="25" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="21" t="s">
         <v>344</v>
       </c>
       <c r="B4" s="15"/>
@@ -6337,7 +6340,7 @@
       <c r="E4" s="15"/>
       <c r="F4" s="15"/>
     </row>
-    <row r="5" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>345</v>
       </c>
@@ -6354,7 +6357,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>349</v>
       </c>
@@ -6371,7 +6374,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>353</v>
       </c>
@@ -6388,7 +6391,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>357</v>
       </c>
@@ -6405,7 +6408,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>359</v>
       </c>
@@ -6422,7 +6425,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>360</v>
       </c>
@@ -6439,7 +6442,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>361</v>
       </c>
@@ -6456,7 +6459,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>362</v>
       </c>
@@ -6473,7 +6476,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>363</v>
       </c>
@@ -6490,7 +6493,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>364</v>
       </c>
@@ -6507,7 +6510,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>365</v>
       </c>
@@ -6524,7 +6527,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>366</v>
       </c>
@@ -6541,7 +6544,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>369</v>
       </c>
@@ -6558,7 +6561,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>372</v>
       </c>
@@ -6575,7 +6578,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>374</v>
       </c>
@@ -6592,7 +6595,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>376</v>
       </c>
@@ -6609,28 +6612,28 @@
         <v>378</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
       <c r="D21" s="8"/>
       <c r="E21" s="8"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
       <c r="D23" s="8"/>
       <c r="E23" s="8"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -6645,10 +6648,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{f42aa342-8706-4288-bd11-ebb85995028c}" enabled="1" method="Standard" siteId="{72f988bf-86f1-41af-91ab-2d7cd011db47}" contentBits="0" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>